<commit_message>
Préstamo: script f_users (FOLIO), flujo BuscarUsuarioFOLIO, Excel con correo de prueba y plazo por defecto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018uFU4P9QkaWXr2H5UAix7x
</commit_message>
<xml_diff>
--- a/prestamo/Prestamos_Ficticios.xlsx
+++ b/prestamo/Prestamos_Ficticios.xlsx
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblPlazos" displayName="tblPlazos" ref="A1:C8" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblPlazos" displayName="tblPlazos" ref="A1:C9" headerRowCount="1">
   <autoFilter ref="A1:C8"/>
   <tableColumns count="3">
     <tableColumn id="1" name="TipoMaterial"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>correo.prueba@uai.cl</t>
+          <t>pablo.salas.marin@uai.cl</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>correo.prueba@uai.cl</t>
+          <t>pablo.salas.marin@uai.cl</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>correo.prueba@uai.cl</t>
+          <t>pablo.salas.marin@uai.cl</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -843,6 +843,11 @@
           <t>SoloSala</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Escribir en TipoMaterial el nombre EXACTO que usa FOLIO (tabla f_mtypes_script, columna name).</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -946,6 +951,21 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>SI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>(cualquier otro tipo)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>28</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>

</xml_diff>